<commit_message>
Add clickable listing links to lead-scan Excel; interval to 10 min
Each listing now carries a url; scan.py writes it as a clickable hyperlink
column in reports/lead_scan.xlsx and prints it in the summary. Background loop
cadence reduced to 10 minutes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xpu1sUMAXpYvcB6L6Wieam
</commit_message>
<xml_diff>
--- a/agentic-gelir-sistemi/reports/lead_scan.xlsx
+++ b/agentic-gelir-sistemi/reports/lead_scan.xlsx
@@ -17,12 +17,19 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -43,14 +50,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -413,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,6 +459,11 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>durum</t>
         </is>
       </c>
@@ -456,7 +471,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-09 11:17:33 UTC</t>
+          <t>2026-07-09 11:22:09 UTC</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -482,7 +497,12 @@
           <t>firmware, embedded, desktop, c#, companion</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.com/Job/firmware-engineer-software-contractor-jobs-SRCH_KO0,37.htm</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
         <is>
           <t>queued</t>
         </is>
@@ -491,7 +511,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-09 11:17:33 UTC</t>
+          <t>2026-07-09 11:22:09 UTC</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -517,7 +537,12 @@
           <t>stm32, firmware, embedded, wpf, desktop, companion</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>https://www.indeed.com/q-Embedded-Firmware-Contract-Engineer-jobs.html</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>queued</t>
         </is>
@@ -526,7 +551,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-07-09 11:17:33 UTC</t>
+          <t>2026-07-09 11:22:09 UTC</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -552,7 +577,12 @@
           <t>esp32, firmware, embedded</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>https://remotive.com/remote/jobs/software-development/senior-embedded-firmware-engineer-4570395</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>queued</t>
         </is>
@@ -561,7 +591,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-09 11:17:33 UTC</t>
+          <t>2026-07-09 11:22:09 UTC</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -587,7 +617,12 @@
           <t>stm32, firmware, embedded, rtos, microcontroller, freertos</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="1" t="inlineStr">
+        <is>
+          <t>https://arc.dev/remote-jobs/firmware</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>queued</t>
         </is>
@@ -596,7 +631,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-07-09 11:17:33 UTC</t>
+          <t>2026-07-09 11:22:09 UTC</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -622,7 +657,12 @@
           <t>esp32, firmware</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="1" t="inlineStr">
+        <is>
+          <t>https://www.upwork.com/freelance-jobs/firmware/</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>queued</t>
         </is>
@@ -631,7 +671,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-09 11:17:33 UTC</t>
+          <t>2026-07-09 11:22:09 UTC</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -657,7 +697,12 @@
           <t>wpf, desktop, c#</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="1" t="inlineStr">
+        <is>
+          <t>https://arc.dev/remote-jobs/wpf</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>queued</t>
         </is>
@@ -666,7 +711,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-07-09 11:17:33 UTC</t>
+          <t>2026-07-09 11:22:09 UTC</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -692,13 +737,27 @@
           <t>desktop</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>https://www.indeed.com/q-c%23-developer-l-remote-jobs.html</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>queued</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId7"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Use Turkey time (TRT, UTC+3) for scan timestamps
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xpu1sUMAXpYvcB6L6Wieam
</commit_message>
<xml_diff>
--- a/agentic-gelir-sistemi/reports/lead_scan.xlsx
+++ b/agentic-gelir-sistemi/reports/lead_scan.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -743,6 +743,286 @@
         </is>
       </c>
       <c r="H8" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-07-09 14:34:44 TRT</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>glassdoor</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Firmware engineer + existing C# companion app maintenance</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>90</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Firmware + companion GUI birlikte — tam niş uyumu (senin moat'ın).</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>firmware, embedded, desktop, c#, companion</t>
+        </is>
+      </c>
+      <c r="G9" s="1" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.com/Job/firmware-engineer-software-contractor-jobs-SRCH_KO0,37.htm</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-07-09 14:34:44 TRT</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>contract-board</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Embedded device with Windows configuration &amp; calibration tool</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>90</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Firmware + companion GUI birlikte — tam niş uyumu (senin moat'ın).</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>stm32, firmware, embedded, wpf, desktop, companion</t>
+        </is>
+      </c>
+      <c r="G10" s="1" t="inlineStr">
+        <is>
+          <t>https://www.indeed.com/q-Embedded-Firmware-Contract-Engineer-jobs.html</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07-09 14:34:44 TRT</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>remotive</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Senior Embedded Firmware Engineer</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>55</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Firmware var ama companion GUI yok — kısmi uyum.</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>esp32, firmware, embedded</t>
+        </is>
+      </c>
+      <c r="G11" s="1" t="inlineStr">
+        <is>
+          <t>https://remotive.com/remote/jobs/software-development/senior-embedded-firmware-engineer-4570395</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-09 14:34:44 TRT</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>arc.dev</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>STM32 firmware contractor (C/C++, FreeRTOS)</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>55</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Firmware var ama companion GUI yok — kısmi uyum.</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>stm32, firmware, embedded, rtos, microcontroller, freertos</t>
+        </is>
+      </c>
+      <c r="G12" s="1" t="inlineStr">
+        <is>
+          <t>https://arc.dev/remote-jobs/firmware</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-07-09 14:34:44 TRT</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>upwork</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ESP32 BLE sensor firmware freelancer</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>55</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Firmware var ama companion GUI yok — kısmi uyum.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>esp32, firmware</t>
+        </is>
+      </c>
+      <c r="G13" s="1" t="inlineStr">
+        <is>
+          <t>https://www.upwork.com/freelance-jobs/firmware/</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07-09 14:34:44 TRT</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>arc.dev</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>WPF desktop application developer</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>40</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Masaüstü/GUI var ama gömülü taraf yok — kısmi uyum.</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>wpf, desktop, c#</t>
+        </is>
+      </c>
+      <c r="G14" s="1" t="inlineStr">
+        <is>
+          <t>https://arc.dev/remote-jobs/wpf</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-07-09 14:34:44 TRT</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Remote full-stack web developer (React/Node)</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>40</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Masaüstü/GUI var ama gömülü taraf yok — kısmi uyum.</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>desktop</t>
+        </is>
+      </c>
+      <c r="G15" s="1" t="inlineStr">
+        <is>
+          <t>https://www.indeed.com/q-c%23-developer-l-remote-jobs.html</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
         <is>
           <t>queued</t>
         </is>
@@ -757,6 +1037,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId14"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Manual lead scan cycle (TRT)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xpu1sUMAXpYvcB6L6Wieam
</commit_message>
<xml_diff>
--- a/agentic-gelir-sistemi/reports/lead_scan.xlsx
+++ b/agentic-gelir-sistemi/reports/lead_scan.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1023,6 +1023,286 @@
         </is>
       </c>
       <c r="H15" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-07-09 14:56:52 TRT</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>glassdoor</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Firmware engineer + existing C# companion app maintenance</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>90</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Firmware + companion GUI birlikte — tam niş uyumu (senin moat'ın).</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>firmware, embedded, desktop, c#, companion</t>
+        </is>
+      </c>
+      <c r="G16" s="1" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.com/Job/firmware-engineer-software-contractor-jobs-SRCH_KO0,37.htm</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-07-09 14:56:52 TRT</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>contract-board</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Embedded device with Windows configuration &amp; calibration tool</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>90</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Firmware + companion GUI birlikte — tam niş uyumu (senin moat'ın).</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>stm32, firmware, embedded, wpf, desktop, companion</t>
+        </is>
+      </c>
+      <c r="G17" s="1" t="inlineStr">
+        <is>
+          <t>https://www.indeed.com/q-Embedded-Firmware-Contract-Engineer-jobs.html</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-07-09 14:56:52 TRT</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>remotive</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Senior Embedded Firmware Engineer</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>55</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Firmware var ama companion GUI yok — kısmi uyum.</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>esp32, firmware, embedded</t>
+        </is>
+      </c>
+      <c r="G18" s="1" t="inlineStr">
+        <is>
+          <t>https://remotive.com/remote/jobs/software-development/senior-embedded-firmware-engineer-4570395</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-07-09 14:56:52 TRT</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>arc.dev</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>STM32 firmware contractor (C/C++, FreeRTOS)</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>55</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Firmware var ama companion GUI yok — kısmi uyum.</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>stm32, firmware, embedded, rtos, microcontroller, freertos</t>
+        </is>
+      </c>
+      <c r="G19" s="1" t="inlineStr">
+        <is>
+          <t>https://arc.dev/remote-jobs/firmware</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-07-09 14:56:52 TRT</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>upwork</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>ESP32 BLE sensor firmware freelancer</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>55</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Firmware var ama companion GUI yok — kısmi uyum.</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>esp32, firmware</t>
+        </is>
+      </c>
+      <c r="G20" s="1" t="inlineStr">
+        <is>
+          <t>https://www.upwork.com/freelance-jobs/firmware/</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-07-09 14:56:52 TRT</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>arc.dev</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>WPF desktop application developer</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>40</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Masaüstü/GUI var ama gömülü taraf yok — kısmi uyum.</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>wpf, desktop, c#</t>
+        </is>
+      </c>
+      <c r="G21" s="1" t="inlineStr">
+        <is>
+          <t>https://arc.dev/remote-jobs/wpf</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-07-09 14:56:52 TRT</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Remote full-stack web developer (React/Node)</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>40</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Masaüstü/GUI var ama gömülü taraf yok — kısmi uyum.</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>desktop</t>
+        </is>
+      </c>
+      <c r="G22" s="1" t="inlineStr">
+        <is>
+          <t>https://www.indeed.com/q-c%23-developer-l-remote-jobs.html</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
         <is>
           <t>queued</t>
         </is>
@@ -1044,6 +1324,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Lead scan cycle (on-demand, TRT)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xpu1sUMAXpYvcB6L6Wieam
</commit_message>
<xml_diff>
--- a/agentic-gelir-sistemi/reports/lead_scan.xlsx
+++ b/agentic-gelir-sistemi/reports/lead_scan.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1303,6 +1303,286 @@
         </is>
       </c>
       <c r="H22" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-07-09 15:20:33 TRT</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>glassdoor</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Firmware engineer + existing C# companion app maintenance</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>90</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Firmware + companion GUI birlikte — tam niş uyumu (senin moat'ın).</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>firmware, embedded, desktop, c#, companion</t>
+        </is>
+      </c>
+      <c r="G23" s="1" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.com/Job/firmware-engineer-software-contractor-jobs-SRCH_KO0,37.htm</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-07-09 15:20:33 TRT</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>contract-board</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Embedded device with Windows configuration &amp; calibration tool</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>90</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Firmware + companion GUI birlikte — tam niş uyumu (senin moat'ın).</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>stm32, firmware, embedded, wpf, desktop, companion</t>
+        </is>
+      </c>
+      <c r="G24" s="1" t="inlineStr">
+        <is>
+          <t>https://www.indeed.com/q-Embedded-Firmware-Contract-Engineer-jobs.html</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-07-09 15:20:33 TRT</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>remotive</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Senior Embedded Firmware Engineer</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>55</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Firmware var ama companion GUI yok — kısmi uyum.</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>esp32, firmware, embedded</t>
+        </is>
+      </c>
+      <c r="G25" s="1" t="inlineStr">
+        <is>
+          <t>https://remotive.com/remote/jobs/software-development/senior-embedded-firmware-engineer-4570395</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-07-09 15:20:33 TRT</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>arc.dev</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>STM32 firmware contractor (C/C++, FreeRTOS)</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>55</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Firmware var ama companion GUI yok — kısmi uyum.</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>stm32, firmware, embedded, rtos, microcontroller, freertos</t>
+        </is>
+      </c>
+      <c r="G26" s="1" t="inlineStr">
+        <is>
+          <t>https://arc.dev/remote-jobs/firmware</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-07-09 15:20:33 TRT</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>upwork</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ESP32 BLE sensor firmware freelancer</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>55</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Firmware var ama companion GUI yok — kısmi uyum.</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>esp32, firmware</t>
+        </is>
+      </c>
+      <c r="G27" s="1" t="inlineStr">
+        <is>
+          <t>https://www.upwork.com/freelance-jobs/firmware/</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-07-09 15:20:33 TRT</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>arc.dev</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>WPF desktop application developer</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>40</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Masaüstü/GUI var ama gömülü taraf yok — kısmi uyum.</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>wpf, desktop, c#</t>
+        </is>
+      </c>
+      <c r="G28" s="1" t="inlineStr">
+        <is>
+          <t>https://arc.dev/remote-jobs/wpf</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-07-09 15:20:33 TRT</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Remote full-stack web developer (React/Node)</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>40</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Masaüstü/GUI var ama gömülü taraf yok — kısmi uyum.</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>desktop</t>
+        </is>
+      </c>
+      <c r="G29" s="1" t="inlineStr">
+        <is>
+          <t>https://www.indeed.com/q-c%23-developer-l-remote-jobs.html</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
         <is>
           <t>queued</t>
         </is>
@@ -1331,6 +1611,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId28"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>